<commit_message>
Make FormulaEngine a workbook calculation engine.
Add FormulaValue coerce/error semantics, absolute/relative and quoted-sheet
refs, AST translate+serialize for formula fill, cross-sheet incremental
recalc stats, formula-bar edit, and raw→numFmt display. Integration tests
via FormulaWorkbookTest and an expanded formulas.xlsx fixture.

Co-authored-by: Tero <terotests@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/gallery/datagrid/fixtures/formulas.xlsx
+++ b/gallery/datagrid/fixtures/formulas.xlsx
@@ -8,7 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Calc" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Other" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Input" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Other" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Errors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="My Sheet" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +452,22 @@
         <f>Other!A1*3</f>
         <v/>
       </c>
+      <c r="I1">
+        <f>$A$1+Input!A1</f>
+        <v/>
+      </c>
+      <c r="J1">
+        <f>SUM(Input!A1:A3)</f>
+        <v/>
+      </c>
+      <c r="K1">
+        <f>IF(J1&gt;50,"large","small")</f>
+        <v/>
+      </c>
+      <c r="L1">
+        <f>'My Sheet'!A1*2</f>
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -461,6 +480,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -477,4 +525,49 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>1/0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IFERROR(A1,123)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
FormulaEngine as workbook calculation engine (coerce, refs, fill, recalc) (#624)
* Extract FormulaFunctions as a unit-testable formula library.

Split FormulaValue and FormulaFunctions out of FormulaEngine so the
engine only parses, tracks deps, and dispatches. Expand coverage
(math/text/logical/info) and add datagrid:formula:test.

Co-authored-by: Tero <terotests@users.noreply.github.com>

* Make FormulaEngine a workbook calculation engine.

Add FormulaValue coerce/error semantics, absolute/relative and quoted-sheet
refs, AST translate+serialize for formula fill, cross-sheet incremental
recalc stats, formula-bar edit, and raw→numFmt display. Integration tests
via FormulaWorkbookTest and an expanded formulas.xlsx fixture.

Co-authored-by: Tero <terotests@users.noreply.github.com>

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Tero <terotests@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/gallery/datagrid/fixtures/formulas.xlsx
+++ b/gallery/datagrid/fixtures/formulas.xlsx
@@ -8,7 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Calc" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Other" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Input" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Other" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Errors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="My Sheet" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +452,22 @@
         <f>Other!A1*3</f>
         <v/>
       </c>
+      <c r="I1">
+        <f>$A$1+Input!A1</f>
+        <v/>
+      </c>
+      <c r="J1">
+        <f>SUM(Input!A1:A3)</f>
+        <v/>
+      </c>
+      <c r="K1">
+        <f>IF(J1&gt;50,"large","small")</f>
+        <v/>
+      </c>
+      <c r="L1">
+        <f>'My Sheet'!A1*2</f>
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -461,6 +480,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -477,4 +525,49 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>1/0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IFERROR(A1,123)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>